<commit_message>
updated excel with complete data
</commit_message>
<xml_diff>
--- a/ahp_comparisons.xlsx
+++ b/ahp_comparisons.xlsx
@@ -5,12 +5,16 @@
   <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="criteria" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="learning" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="friends" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="school_life" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="vocational_training" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="college_prep" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="music_classes" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="18">
   <si>
     <t xml:space="preserve">l</t>
   </si>
@@ -90,6 +94,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -127,7 +132,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -144,6 +149,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFB2B2B2"/>
         <bgColor rgb="FF999999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCCC"/>
+        <bgColor rgb="FFCCCCFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -181,36 +192,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -239,9 +258,9 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFCCCCCC"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FFB2B2B2"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
@@ -400,131 +419,131 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.08"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="1" t="n">
+      <c r="B2" s="3"/>
+      <c r="C2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1" t="n">
+      <c r="E2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="2" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="1" t="n">
+      <c r="B3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="1" t="n">
+      <c r="F3" s="4"/>
+      <c r="G3" s="2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="1" t="n">
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="1" t="n">
+      <c r="B6" s="5"/>
+      <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="1" t="n">
+      <c r="E6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="2" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="n">
+      <c r="B7" s="5"/>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="2"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -545,50 +564,50 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="0" t="n">
+      <c r="C3" s="7"/>
+      <c r="D3" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -606,9 +625,307 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.51"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.64"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9"/>
+      <c r="D4" s="7"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
updated row and column names to be identical
</commit_message>
<xml_diff>
--- a/ahp_comparisons.xlsx
+++ b/ahp_comparisons.xlsx
@@ -26,25 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="18">
-  <si>
-    <t xml:space="preserve">l</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mc</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="9">
   <si>
     <t xml:space="preserve">learning</t>
   </si>
@@ -52,25 +34,16 @@
     <t xml:space="preserve">friends</t>
   </si>
   <si>
-    <t xml:space="preserve">school life</t>
+    <t xml:space="preserve">school_life</t>
   </si>
   <si>
-    <t xml:space="preserve">vocational training</t>
+    <t xml:space="preserve">vocational_training</t>
   </si>
   <si>
-    <t xml:space="preserve">college prep</t>
+    <t xml:space="preserve">college_prep</t>
   </si>
   <si>
-    <t xml:space="preserve">music classes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c</t>
+    <t xml:space="preserve">music_classes</t>
   </si>
   <si>
     <t xml:space="preserve">lower merian (a)</t>
@@ -89,7 +62,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -116,6 +89,11 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -192,7 +170,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -205,19 +183,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -420,6 +402,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -430,24 +413,24 @@
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="B2" s="4"/>
       <c r="C2" s="2" t="n">
         <v>4</v>
       </c>
@@ -466,54 +449,54 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="B3" s="5"/>
+      <c r="C3" s="4"/>
       <c r="D3" s="2" t="n">
         <v>7</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="4"/>
+      <c r="F3" s="5"/>
       <c r="G3" s="2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+        <v>2</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="5"/>
       <c r="D5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="E5" s="4"/>
       <c r="F5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="6"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5"/>
+        <v>4</v>
+      </c>
+      <c r="B6" s="6"/>
       <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
@@ -523,16 +506,16 @@
       <c r="E6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="4"/>
       <c r="G6" s="2" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="5"/>
+        <v>5</v>
+      </c>
+      <c r="B7" s="6"/>
       <c r="C7" s="2" t="n">
         <v>1</v>
       </c>
@@ -542,8 +525,8 @@
       <c r="E7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="3"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -570,44 +553,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="7"/>
+      <c r="C3" s="8"/>
       <c r="D3" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="7"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -633,20 +616,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="8"/>
       <c r="C2" s="1" t="n">
         <v>1</v>
       </c>
@@ -656,19 +639,19 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="7"/>
+      <c r="C3" s="8"/>
       <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
@@ -676,7 +659,7 @@
       <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -698,24 +681,26 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.38"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="8"/>
       <c r="C2" s="1" t="n">
         <v>5</v>
       </c>
@@ -725,15 +710,15 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="9"/>
+        <v>7</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
@@ -741,7 +726,7 @@
       <c r="C4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -764,20 +749,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="8"/>
       <c r="C2" s="1" t="n">
         <v>9</v>
       </c>
@@ -787,21 +772,21 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="9"/>
+        <v>7</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="9"/>
+        <v>8</v>
+      </c>
+      <c r="B4" s="10"/>
       <c r="C4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -824,46 +809,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="9"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="7"/>
+      <c r="C3" s="8"/>
       <c r="D3" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="7"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -886,20 +871,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="8"/>
       <c r="C2" s="1" t="n">
         <v>6</v>
       </c>
@@ -909,21 +894,21 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="9"/>
+        <v>7</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="9"/>
+        <v>8</v>
+      </c>
+      <c r="B4" s="10"/>
       <c r="C4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>